<commit_message>
Generate every sheet of the LCOS Signal Manager plan from live data, because patching the workbook had lost its block index and watch lists.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/wiring/lcos/lcos_signal_manager_config_plan.xlsx
+++ b/docs/wiring/lcos/lcos_signal_manager_config_plan.xlsx
@@ -9,11 +9,10 @@
   <sheets>
     <sheet name="Legend" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="By Signal" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Turnout Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Block Index" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Turnout Index" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'By Signal'!$A$1:$P$37</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -31,20 +30,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -61,7 +54,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,27 +420,209 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>LCOS Signal Manager ports (regen 2026-09-08)</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LCOS Signal Manager config plan</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OU1=0-7, OU2=8-15, OU3=16-23, OU4=24-31. C13: motors OU2; 8LA/8LB Digicon OU3.</t>
+          <t>Generated 2026-10-31 by build_lcos_signal_manager_plan.py from live data.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Switch 7/11/13 TWOSENSOR. Switch 7/9/11 on Node 13 OU:2.</t>
+      <c r="A3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sort: Node → LCOS Signal index → Mast/Head</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ports: flat index for Signal Manager Port A/B/C pickers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OU1 pins 1–8 → ports 0–7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OU2 pins 1–8 → ports 8–15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OU3 → 16–23, OU4 → 24–31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Formula: port = (OU - 1) * 8 + (pin - 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Aspect map: Port A = STOP (R), Port B = APPROACH (Y), Port C = CLEAR (G). Field wiring is Stop, Approach, Clear on consecutive increasing ports (R then Y then G).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Turnout polarity: Main = Normal (closed); Diverged = Reverse (thrown). Intermediates 2035/2036 have no plant turnout (—).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Stock Signal Manager sentence: CLEAR if aligned {Main|Diverged} or set aspect {Stop|Approach}. Occupied blocks still force STOP. 2-head top = Main/Stop; bottom = Diverged/Stop (unused disc stays red). Diverge dwarfs = Diverged/Stop. Balloon 2035/2036 = — / Approach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  C13: motors on OU2; 8LA/8LB Digicon on OU3. Switch 7/11/13 are TWOSENSOR. Switch 7/9/11 are on Node 13 OU2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Turnouts / Blocks Node:id match JMRI comments:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Node: N Turnout: T   (T is 0-based LCOS turnout index on that client)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Node: N Block: B     (B is 1-based in comments; LCOS SM checkbox = B-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Block groups (route-dependent ABS intent):</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Throat A,B = two blocks before the facing-point entrance</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Main C,D   = two blocks on the normal / MAIN path</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Diverge E,F = two blocks on the DIVERGED path</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  When a leg has only one detector, only one entry is listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cross-node: if Node:id is not this signal client, subscribe that node and use Remote 8–15</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (remote checkbox = 8 + neighbor local idx). Confirm peer order in LCOS object listen list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sources: docs/wiring/signals/signal_wiring.csv, docs/wiring/lcos/lcos_signal_logic.csv,</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  docs/wiring/lcos/lcos_signal_plan_notes.csv, jmri/layouts/hart/output/tables.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Plant block assignments are the intended ABS watch lists for native LCOS / proposed route UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Stock Signal Manager cannot gate main vs diverge blocks on one head — prefer one head per entrance where route-dependent logic matters.</t>
         </is>
       </c>
     </row>
@@ -462,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:W37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +718,42 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Signal role</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Turnout polarity</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>OR aspect</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Turnouts (name + Node:id)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Blocks throat A,B (before)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Blocks main C,D (normal)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Blocks diverge E,F</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Boundary note</t>
         </is>
       </c>
     </row>
@@ -613,7 +823,42 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>east_lead</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
           <t>Switch 35 (Node: 1 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>BS East Lead (Node: 1 Block: 7; LCOS idx 6) | BS Switch 35b (Node: 1 Block: 5; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>BS Switch 35b (Node: 1 Block: 5; LCOS idx 4) | BS Switch 35a (Node: 1 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>BS Switch 35b (Node: 1 Block: 5; LCOS idx 4) | BS West Main Ext (Node: 1 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>D=Track East Lead west lower</t>
         </is>
       </c>
     </row>
@@ -683,7 +928,42 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>east_lead</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>Switch 35 (Node: 1 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>BS East Lead (Node: 1 Block: 7; LCOS idx 6) | BS Switch 35b (Node: 1 Block: 5; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>BS Switch 35b (Node: 1 Block: 5; LCOS idx 4) | BS Switch 35a (Node: 1 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>BS Switch 35b (Node: 1 Block: 5; LCOS idx 4) | BS West Main Ext (Node: 1 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>D=Track East Lead west lower</t>
         </is>
       </c>
     </row>
@@ -753,7 +1033,42 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>west_main_ext</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>Switch 35 (Node: 1 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>BS West Main Ext (Node: 1 Block: 8; LCOS idx 7) | BS Switch 35a (Node: 1 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>BS Switch 35a (Node: 1 Block: 6; LCOS idx 5) | BS Switch 35b (Node: 1 Block: 5; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>BS Switch 35a (Node: 1 Block: 6; LCOS idx 5) | BS East Lead (Node: 1 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>A=Track West Main Ext west upper</t>
         </is>
       </c>
     </row>
@@ -823,7 +1138,42 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>west_main_ext</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>Switch 35 (Node: 1 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>BS West Main Ext (Node: 1 Block: 8; LCOS idx 7) | BS Switch 35a (Node: 1 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>BS Switch 35a (Node: 1 Block: 6; LCOS idx 5) | BS Switch 35b (Node: 1 Block: 5; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>BS Switch 35a (Node: 1 Block: 6; LCOS idx 5) | BS East Lead (Node: 1 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>A=Track West Main Ext west upper</t>
         </is>
       </c>
     </row>
@@ -893,7 +1243,38 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
+          <t>mckeesport</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
           <t>Switch 37 (Node: 1 Turnout: 1; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>BS McKeesport (Node: 1 Block: 2; LCOS idx 1) | BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2) | BS McKeesport (Node: 1 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>C=Track McKeesport (boundary at turnout); icon deg 270 faces west</t>
         </is>
       </c>
     </row>
@@ -963,7 +1344,38 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>mckeesport</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
           <t>Switch 37 (Node: 1 Turnout: 1; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>BS McKeesport (Node: 1 Block: 2; LCOS idx 1) | BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2) | BS McKeesport (Node: 1 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>C=Track McKeesport (boundary at turnout); icon deg 270 faces west</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1445,38 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>k2</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
           <t>Switch 37 (Node: 1 Turnout: 1; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2) | BS McKeesport (Node: 1 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>B=Track K-2 stub block (detector Block 1-3 shared with Track 37)</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1546,42 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>main_west_entrance</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
           <t>Switch 23 (Node: 12 Turnout: 4; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>BS Main West (Node: 2 Block: 1; LCOS idx 0) | BS Switch 23a (Node: 12 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>BS Switch 23a (Node: 12 Block: 4; LCOS idx 3) | BS Switch 23b (Node: 12 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>BS Switch 23a (Node: 12 Block: 4; LCOS idx 3) | BS S-R (Node: 2 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>A=Track Main West west upper</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1651,42 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>ext_entrance</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
           <t>Switch 23 (Node: 12 Turnout: 4; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BS West Main Ext (Node: 1 Block: 8; LCOS idx 7) | BS Switch 23b (Node: 12 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>BS Switch 23b (Node: 12 Block: 6; LCOS idx 5) | BS Main West (Node: 2 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>BS Switch 23b (Node: 12 Block: 6; LCOS idx 5) | BS S-R (Node: 2 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>B=Track West Main Ext east upper</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1756,38 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
+          <t>siding_entrance</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
           <t>Switch 23 (Node: 12 Turnout: 4; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>BS S-R (Node: 2 Block: 8; LCOS idx 7) | BS Switch 23a (Node: 12 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>BS Switch 23a (Node: 12 Block: 4; LCOS idx 3) | BS Main West (Node: 2 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>D=Track S-R west lower</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1857,42 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
+          <t>main_west_entrance</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
           <t>Switch 23 (Node: 12 Turnout: 4; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>BS Main West (Node: 2 Block: 1; LCOS idx 0) | BS Switch 23a (Node: 12 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>BS Switch 23a (Node: 12 Block: 4; LCOS idx 3) | BS Switch 23b (Node: 12 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>BS Switch 23a (Node: 12 Block: 4; LCOS idx 3) | BS S-R (Node: 2 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>A=Track Main West west upper</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1962,42 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
+          <t>ext_entrance</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
           <t>Switch 23 (Node: 12 Turnout: 4; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>BS West Main Ext (Node: 1 Block: 8; LCOS idx 7) | BS Switch 23b (Node: 12 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>BS Switch 23b (Node: 12 Block: 6; LCOS idx 5) | BS Main West (Node: 2 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>BS Switch 23b (Node: 12 Block: 6; LCOS idx 5) | BS S-R (Node: 2 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>B=Track West Main Ext east upper</t>
         </is>
       </c>
     </row>
@@ -1453,7 +2067,38 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
+          <t>main_exit</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
           <t>Switch 5 (Node: 4 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>BS Switch 5 (Node: 4 Block: 5; LCOS idx 4) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>BS Switch 5 (Node: 4 Block: 5; LCOS idx 4) | BS Scale (Node: 4 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>B=Track East Main Ext continuing</t>
         </is>
       </c>
     </row>
@@ -1523,7 +2168,38 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
+          <t>main_exit</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
           <t>Switch 5 (Node: 4 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>BS Switch 5 (Node: 4 Block: 5; LCOS idx 4) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>BS Switch 5 (Node: 4 Block: 5; LCOS idx 4) | BS Scale (Node: 4 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>B=Track East Main Ext continuing</t>
         </is>
       </c>
     </row>
@@ -1593,7 +2269,34 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
+          <t>diverge_exit</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
           <t>Switch 5 (Node: 4 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>BS Switch 5 (Node: 4 Block: 5; LCOS idx 4) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>C=Track Scale / east upper face; 1-head IH434</t>
         </is>
       </c>
     </row>
@@ -1663,7 +2366,34 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
+          <t>main_exit</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
           <t>Switch 3 (Node: 4 Turnout: 1; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>BS Switch 3 (Node: 4 Block: 1; LCOS idx 0) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>B=Track W-1 continuing</t>
         </is>
       </c>
     </row>
@@ -1733,7 +2463,34 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
+          <t>diverge_exit</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
           <t>Switch 3 (Node: 4 Turnout: 1; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>BS Switch 3 (Node: 4 Block: 1; LCOS idx 0) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>C=Track W-2 diverge</t>
         </is>
       </c>
     </row>
@@ -1803,7 +2560,38 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
+          <t>throat_east</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
           <t>Switch 1 (Node: 4 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>BS Main West (Node: 2 Block: 1; LCOS idx 0) | BS Switch 1 (Node: 4 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>BS Switch 1 (Node: 4 Block: 2; LCOS idx 1) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>A=Track Main West; east face of Brick</t>
         </is>
       </c>
     </row>
@@ -1873,7 +2661,38 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
+          <t>throat_east</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
           <t>Switch 1 (Node: 4 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>BS Main West (Node: 2 Block: 1; LCOS idx 0) | BS Switch 1 (Node: 4 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>BS Switch 1 (Node: 4 Block: 2; LCOS idx 1) | BS Brick-Plane (Node: 4 Block: 6; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>A=Track Main West; east face of Brick</t>
         </is>
       </c>
     </row>
@@ -1943,7 +2762,38 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
+          <t>mckees_rocks</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
           <t>Switch 39 (Node: 1 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0) | BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3) | BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>C=Track McKees Rocks (boundary at turnout); icon deg 270 faces west</t>
         </is>
       </c>
     </row>
@@ -2006,8 +2856,43 @@
           <t>C11-OU3-6</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>McKeesport intermediate</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>BS McKeesport (Node: 1 Block: 2; LCOS idx 1)</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>BS McKeesport (Node: 1 Block: 2; LCOS idx 1) | BS Switch 37 / BS K-2 (Node: 1 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Track McKeesport intermediate; CATS (61</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2068,8 +2953,43 @@
           <t>C11-OU2-7</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>McKees Rocks intermediate</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0) | BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>Track McKees Rocks intermediate; CATS (60</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2137,7 +3057,38 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
+          <t>mckees_rocks</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
           <t>Switch 39 (Node: 1 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0) | BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3) | BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>C=Track McKees Rocks (boundary at turnout); icon deg 270 faces west</t>
         </is>
       </c>
     </row>
@@ -2207,7 +3158,38 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
+          <t>k1</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
           <t>Switch 39 (Node: 1 Turnout: 2; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>BS Switch 39 / BS K-1 (Node: 1 Block: 4; LCOS idx 3) | BS McKees Rocks (Node: 1 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>B=Track K-1 stub block (detector Block 1-4 shared with Track 39)</t>
         </is>
       </c>
     </row>
@@ -2277,7 +3259,42 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
+          <t>east_lead</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
           <t>Switch 33 (Node: 12 Turnout: 5; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>BS East Lead (Node: 1 Block: 7; LCOS idx 6) | BS Switch 33 (Node: 12 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS Main East (Node: 2 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS Switch 31 (Node: 12 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>A=Track East Lead east of 112</t>
         </is>
       </c>
     </row>
@@ -2347,7 +3364,42 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
+          <t>east_lead</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
           <t>Switch 33 (Node: 12 Turnout: 5; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>BS East Lead (Node: 1 Block: 7; LCOS idx 6) | BS Switch 33 (Node: 12 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS Main East (Node: 2 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS Switch 31 (Node: 12 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>A=Track East Lead east of 112</t>
         </is>
       </c>
     </row>
@@ -2417,7 +3469,42 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
+          <t>ladder</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
           <t>Switch 31 (Node: 12 Turnout: 3; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>BS Switch 31 (Node: 12 Block: 7; LCOS idx 6) | BS Switch 29 (Node: 12 Block: 5; LCOS idx 4)</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>BS Switch 31 (Node: 12 Block: 7; LCOS idx 6) | BS Switch 33 (Node: 12 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>BS Switch 31 (Node: 12 Block: 7; LCOS idx 6) | BS Switch 25 (Node: 12 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>C=Track 29 ladder leg; governs ladder move into Track 31</t>
         </is>
       </c>
     </row>
@@ -2487,7 +3574,38 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
+          <t>main_east</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
           <t>Switch 33 (Node: 12 Turnout: 5; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>BS Main East (Node: 2 Block: 3; LCOS idx 2) | BS Switch 33 (Node: 12 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS East Lead (Node: 1 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>C=Track Main East diverge</t>
         </is>
       </c>
     </row>
@@ -2557,7 +3675,38 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
+          <t>main_east</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
           <t>Switch 33 (Node: 12 Turnout: 5; LCOS idx 5)</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>BS Main East (Node: 2 Block: 3; LCOS idx 2) | BS Switch 33 (Node: 12 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>BS Switch 33 (Node: 12 Block: 8; LCOS idx 7) | BS East Lead (Node: 1 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>C=Track Main East diverge</t>
         </is>
       </c>
     </row>
@@ -2627,7 +3776,42 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
+          <t>west_cluster</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS East Main Ext (Node: 4 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Scale (Node: 4 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>Scale|Switch 7 eastbound; not TO117 A</t>
         </is>
       </c>
     </row>
@@ -2697,7 +3881,42 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
+          <t>west_cluster</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS East Main Ext (Node: 4 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Scale (Node: 4 Block: 8; LCOS idx 7)</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>Scale|Switch 7 eastbound; not TO117 A</t>
         </is>
       </c>
     </row>
@@ -2767,7 +3986,38 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
+          <t>east_barn</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Barn (Node: 13 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>B=Track Barn east upper</t>
         </is>
       </c>
     </row>
@@ -2837,7 +4087,42 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
+          <t>west_lower</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>BS Switch 7b (Node: 13 Block: 4; LCOS idx 3) | BS East Main Ext (Node: 4 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Barn (Node: 13 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>D=Track East Main Ext west lower</t>
         </is>
       </c>
     </row>
@@ -2907,7 +4192,42 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
+          <t>west_lower</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>BS Switch 7b (Node: 13 Block: 4; LCOS idx 3) | BS East Main Ext (Node: 4 Block: 7; LCOS idx 6)</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Barn (Node: 13 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>D=Track East Main Ext west lower</t>
         </is>
       </c>
     </row>
@@ -2977,7 +4297,42 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
+          <t>east_main</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Main East (Node: 2 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Barn (Node: 13 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>C=Track Main East east lower</t>
         </is>
       </c>
     </row>
@@ -3047,12 +4402,46 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
+          <t>east_main</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Diverged</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Stop</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
           <t>Switch 7 (Node: 13 Turnout: 0; LCOS idx 0)</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Switch 7b (Node: 13 Block: 4; LCOS idx 3)</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Main East (Node: 2 Block: 3; LCOS idx 2)</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>BS Switch 7 (Node: 13 Block: 3; LCOS idx 2) | BS Barn (Node: 13 Block: 1; LCOS idx 0)</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>C=Track Main East east lower</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3063,26 +4452,1056 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Node</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>LCOS idx (0-7)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>JMRI Block #</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Node:id</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>BS name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>BS McKees Rocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BS McKeesport</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BS Switch 37 / BS K-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BS Switch 39 / BS K-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BS Switch 35b</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 6</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BS Switch 35a</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 7</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BS East Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Node: 1 Block: 8</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BS West Main Ext</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BS Main West</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 3</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BS Main East</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 4</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BS S-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 5</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BS S-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 6</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BS S-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 7</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BS S-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Node: 2 Block: 8</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BS S-R</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Node: 3 Block: 1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BS Switch 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Node: 3 Block: 2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>BS Switch 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Node: 3 Block: 3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>BS Switch 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Node: 3 Block: 5</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BS Switch 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Node: 3 Block: 7</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>BS Switch 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>BS Switch 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BS Switch 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>BS W-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 4</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BS W-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 5</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BS Switch 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 6</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BS Brick-Plane</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 7</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BS East Main Ext</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Node: 4 Block: 8</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BS Scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BS Switch 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BS Switch 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 4</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>BS Switch 23a</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 5</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>BS Switch 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 6</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>BS Switch 23b</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 7</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>BS Switch 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>7</v>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Node: 12 Block: 8</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>BS Switch 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 1</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>BS Barn</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 2</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>BS Switch 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 3</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>BS Switch 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 4</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>BS Switch 7b</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 5</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>BS EH-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" t="n">
+        <v>6</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 6</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BS EH-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" t="n">
+        <v>7</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 7</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>BS EH-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>7</v>
+      </c>
+      <c r="C44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Node: 13 Block: 8</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>BS Switch 9</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Node</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>LCOS idx</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Node:id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Switch name</t>
         </is>

</xml_diff>